<commit_message>
v3.1: fix - 2026/07/28
</commit_message>
<xml_diff>
--- a/resources/M626/spc_cpk_detail.xlsx
+++ b/resources/M626/spc_cpk_detail.xlsx
@@ -847,10 +847,10 @@
         <v>46230.72840277778</v>
       </c>
       <c r="J2">
-        <v>1.783316479126941</v>
+        <v>1.783316479126942</v>
       </c>
       <c r="K2">
-        <v>1.783316479126941</v>
+        <v>1.783316479126942</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1232,10 +1232,10 @@
         <v>46227.67450231482</v>
       </c>
       <c r="J13">
-        <v>2.610324736578182</v>
+        <v>2.610324736578181</v>
       </c>
       <c r="K13">
-        <v>2.610324736578182</v>
+        <v>2.610324736578181</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1302,10 +1302,10 @@
         <v>46227.67450231482</v>
       </c>
       <c r="J15">
-        <v>2.610324736578182</v>
+        <v>2.610324736578181</v>
       </c>
       <c r="K15">
-        <v>2.610324736578182</v>
+        <v>2.610324736578181</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -2002,10 +2002,10 @@
         <v>46184.60541666667</v>
       </c>
       <c r="J35">
-        <v>1.60078530526187</v>
+        <v>1.600785305261871</v>
       </c>
       <c r="K35">
-        <v>1.60078530526187</v>
+        <v>1.600785305261871</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2912,10 +2912,10 @@
         <v>46191.72753472222</v>
       </c>
       <c r="J61">
-        <v>1.522077432746186</v>
+        <v>1.522077432746187</v>
       </c>
       <c r="K61">
-        <v>1.522077432746186</v>
+        <v>1.522077432746187</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -3017,10 +3017,10 @@
         <v>46191.72753472222</v>
       </c>
       <c r="J64">
-        <v>2.621307957323171</v>
+        <v>2.621307957323172</v>
       </c>
       <c r="K64">
-        <v>2.621307957323171</v>
+        <v>2.621307957323172</v>
       </c>
     </row>
     <row r="65" spans="1:11">
@@ -3857,10 +3857,10 @@
         <v>46191.74302083333</v>
       </c>
       <c r="J88">
-        <v>1.7003357646203</v>
+        <v>1.700335764620301</v>
       </c>
       <c r="K88">
-        <v>1.7003357646203</v>
+        <v>1.700335764620301</v>
       </c>
     </row>
     <row r="89" spans="1:11">
@@ -3927,10 +3927,10 @@
         <v>46191.74302083333</v>
       </c>
       <c r="J90">
-        <v>1.7003357646203</v>
+        <v>1.700335764620301</v>
       </c>
       <c r="K90">
-        <v>1.7003357646203</v>
+        <v>1.700335764620301</v>
       </c>
     </row>
     <row r="91" spans="1:11">
@@ -4977,10 +4977,10 @@
         <v>46183.9808912037</v>
       </c>
       <c r="J120">
-        <v>1.549513971338662</v>
+        <v>1.549513971338663</v>
       </c>
       <c r="K120">
-        <v>1.549513971338662</v>
+        <v>1.549513971338663</v>
       </c>
     </row>
     <row r="121" spans="1:11">
@@ -5082,10 +5082,10 @@
         <v>46183.9808912037</v>
       </c>
       <c r="J123">
-        <v>1.549513971338662</v>
+        <v>1.549513971338663</v>
       </c>
       <c r="K123">
-        <v>1.549513971338662</v>
+        <v>1.549513971338663</v>
       </c>
     </row>
     <row r="124" spans="1:11">
@@ -5187,10 +5187,10 @@
         <v>46175.90008101852</v>
       </c>
       <c r="J126">
-        <v>1.907125675379762</v>
+        <v>1.907125675379763</v>
       </c>
       <c r="K126">
-        <v>1.907125675379762</v>
+        <v>1.907125675379763</v>
       </c>
     </row>
     <row r="127" spans="1:11">
@@ -5292,10 +5292,10 @@
         <v>46175.90008101852</v>
       </c>
       <c r="J129">
-        <v>1.907125675379762</v>
+        <v>1.907125675379763</v>
       </c>
       <c r="K129">
-        <v>1.907125675379762</v>
+        <v>1.907125675379763</v>
       </c>
     </row>
     <row r="130" spans="1:11">
@@ -7077,10 +7077,10 @@
         <v>46176.74538194444</v>
       </c>
       <c r="J180">
-        <v>2.75604192212703</v>
+        <v>2.756041922127031</v>
       </c>
       <c r="K180">
-        <v>2.75604192212703</v>
+        <v>2.756041922127031</v>
       </c>
     </row>
     <row r="181" spans="1:11">
@@ -7147,10 +7147,10 @@
         <v>46176.74538194444</v>
       </c>
       <c r="J182">
-        <v>2.75604192212703</v>
+        <v>2.756041922127031</v>
       </c>
       <c r="K182">
-        <v>2.75604192212703</v>
+        <v>2.756041922127031</v>
       </c>
     </row>
     <row r="183" spans="1:11">
@@ -7917,10 +7917,10 @@
         <v>46195.25652777778</v>
       </c>
       <c r="J204">
-        <v>1.943192331634054</v>
+        <v>1.943192331634055</v>
       </c>
       <c r="K204">
-        <v>1.943192331634054</v>
+        <v>1.943192331634055</v>
       </c>
     </row>
     <row r="205" spans="1:11">
@@ -8022,10 +8022,10 @@
         <v>46195.25652777778</v>
       </c>
       <c r="J207">
-        <v>1.943192331634054</v>
+        <v>1.943192331634055</v>
       </c>
       <c r="K207">
-        <v>1.943192331634054</v>
+        <v>1.943192331634055</v>
       </c>
     </row>
     <row r="208" spans="1:11">
@@ -8407,10 +8407,10 @@
         <v>46187.56212962963</v>
       </c>
       <c r="J218">
-        <v>3.124467950828476</v>
+        <v>3.124467950828475</v>
       </c>
       <c r="K218">
-        <v>3.124467950828476</v>
+        <v>3.124467950828475</v>
       </c>
     </row>
     <row r="219" spans="1:11">
@@ -9492,10 +9492,10 @@
         <v>46179.84344907408</v>
       </c>
       <c r="J249">
-        <v>2.522126018705464</v>
+        <v>2.522126018705463</v>
       </c>
       <c r="K249">
-        <v>2.522126018705464</v>
+        <v>2.522126018705463</v>
       </c>
     </row>
     <row r="250" spans="1:11">
@@ -10332,10 +10332,10 @@
         <v>46183.84069444444</v>
       </c>
       <c r="J273">
-        <v>3.473296225913956</v>
+        <v>3.473296225913955</v>
       </c>
       <c r="K273">
-        <v>3.473296225913956</v>
+        <v>3.473296225913955</v>
       </c>
     </row>
     <row r="274" spans="1:11">
@@ -10612,10 +10612,10 @@
         <v>46207.44892361111</v>
       </c>
       <c r="J281">
-        <v>1.978853450574098</v>
+        <v>1.978853450574099</v>
       </c>
       <c r="K281">
-        <v>1.978853450574098</v>
+        <v>1.978853450574099</v>
       </c>
     </row>
     <row r="282" spans="1:11">
@@ -11277,10 +11277,10 @@
         <v>46203.94153935185</v>
       </c>
       <c r="J300">
-        <v>4.318794497148454</v>
+        <v>4.318794497148455</v>
       </c>
       <c r="K300">
-        <v>4.318794497148454</v>
+        <v>4.318794497148455</v>
       </c>
     </row>
     <row r="301" spans="1:11">
@@ -11487,10 +11487,10 @@
         <v>46175.98122685185</v>
       </c>
       <c r="J306">
-        <v>4.758989576321312</v>
+        <v>4.758989576321313</v>
       </c>
       <c r="K306">
-        <v>4.758989576321312</v>
+        <v>4.758989576321313</v>
       </c>
     </row>
     <row r="307" spans="1:11">
@@ -11977,10 +11977,10 @@
         <v>46203.94153935185</v>
       </c>
       <c r="J320">
-        <v>1.800625414669072</v>
+        <v>1.800625414669073</v>
       </c>
       <c r="K320">
-        <v>1.800625414669072</v>
+        <v>1.800625414669073</v>
       </c>
     </row>
     <row r="321" spans="1:11">
@@ -12047,10 +12047,10 @@
         <v>46180.88512731482</v>
       </c>
       <c r="J322">
-        <v>1.979439625650374</v>
+        <v>1.979439625650375</v>
       </c>
       <c r="K322">
-        <v>1.979439625650374</v>
+        <v>1.979439625650375</v>
       </c>
     </row>
     <row r="323" spans="1:11">
@@ -12082,10 +12082,10 @@
         <v>46183.84069444444</v>
       </c>
       <c r="J323">
-        <v>2.13289939599393</v>
+        <v>2.132899395993929</v>
       </c>
       <c r="K323">
-        <v>2.13289939599393</v>
+        <v>2.132899395993929</v>
       </c>
     </row>
     <row r="324" spans="1:11">
@@ -12572,10 +12572,10 @@
         <v>46205.77965277778</v>
       </c>
       <c r="J337">
-        <v>2.013994314162455</v>
+        <v>2.013994314162456</v>
       </c>
       <c r="K337">
-        <v>2.013994314162455</v>
+        <v>2.013994314162456</v>
       </c>
     </row>
     <row r="338" spans="1:11">
@@ -13447,10 +13447,10 @@
         <v>46180.86203703703</v>
       </c>
       <c r="J362">
-        <v>6.429124494415824</v>
+        <v>6.429124494415822</v>
       </c>
       <c r="K362">
-        <v>6.429124494415824</v>
+        <v>6.429124494415822</v>
       </c>
     </row>
     <row r="363" spans="1:11">
@@ -13552,10 +13552,10 @@
         <v>46174.94690972222</v>
       </c>
       <c r="J365">
-        <v>7.589856339205541</v>
+        <v>7.589856339205542</v>
       </c>
       <c r="K365">
-        <v>7.589856339205541</v>
+        <v>7.589856339205542</v>
       </c>
     </row>
     <row r="366" spans="1:11">
@@ -13937,10 +13937,10 @@
         <v>46203.91032407407</v>
       </c>
       <c r="J376">
-        <v>6.710504533536466</v>
+        <v>6.710504533536464</v>
       </c>
       <c r="K376">
-        <v>6.710504533536466</v>
+        <v>6.710504533536464</v>
       </c>
     </row>
     <row r="377" spans="1:11">
@@ -13972,10 +13972,10 @@
         <v>46204.45003472222</v>
       </c>
       <c r="J377">
-        <v>5.867270425380308</v>
+        <v>5.867270425380309</v>
       </c>
       <c r="K377">
-        <v>5.867270425380308</v>
+        <v>5.867270425380309</v>
       </c>
     </row>
     <row r="378" spans="1:11">
@@ -14007,10 +14007,10 @@
         <v>46205.74840277778</v>
       </c>
       <c r="J378">
-        <v>5.002728289455207</v>
+        <v>5.002728289455206</v>
       </c>
       <c r="K378">
-        <v>5.002728289455207</v>
+        <v>5.002728289455206</v>
       </c>
     </row>
     <row r="379" spans="1:11">
@@ -14322,10 +14322,10 @@
         <v>46175.99747685185</v>
       </c>
       <c r="J387">
-        <v>2.340653643500904</v>
+        <v>2.340653643500905</v>
       </c>
       <c r="K387">
-        <v>2.340653643500904</v>
+        <v>2.340653643500905</v>
       </c>
     </row>
     <row r="388" spans="1:11">
@@ -14392,10 +14392,10 @@
         <v>46177.64208333333</v>
       </c>
       <c r="J389">
-        <v>2.292708884922962</v>
+        <v>2.292708884922961</v>
       </c>
       <c r="K389">
-        <v>2.292708884922962</v>
+        <v>2.292708884922961</v>
       </c>
     </row>
     <row r="390" spans="1:11">
@@ -14987,10 +14987,10 @@
         <v>46207.33239583333</v>
       </c>
       <c r="J406">
-        <v>5.126003391461595</v>
+        <v>5.126003391461596</v>
       </c>
       <c r="K406">
-        <v>5.126003391461595</v>
+        <v>5.126003391461596</v>
       </c>
     </row>
     <row r="407" spans="1:11">
@@ -15127,10 +15127,10 @@
         <v>46177.64207175926</v>
       </c>
       <c r="J410">
-        <v>4.123180426844028</v>
+        <v>4.123180426844027</v>
       </c>
       <c r="K410">
-        <v>4.123180426844028</v>
+        <v>4.123180426844027</v>
       </c>
     </row>
     <row r="411" spans="1:11">
@@ -15617,10 +15617,10 @@
         <v>46207.33239583333</v>
       </c>
       <c r="J424">
-        <v>3.09010363110375</v>
+        <v>3.090103631103751</v>
       </c>
       <c r="K424">
-        <v>3.09010363110375</v>
+        <v>3.090103631103751</v>
       </c>
     </row>
     <row r="425" spans="1:11">
@@ -15897,10 +15897,10 @@
         <v>46178.9991087963</v>
       </c>
       <c r="J432">
-        <v>4.502718598162202</v>
+        <v>4.502718598162201</v>
       </c>
       <c r="K432">
-        <v>4.502718598162202</v>
+        <v>4.502718598162201</v>
       </c>
     </row>
     <row r="433" spans="1:11">
@@ -16527,10 +16527,10 @@
         <v>46175.99745370371</v>
       </c>
       <c r="J450">
-        <v>3.041971341412588</v>
+        <v>3.041971341412587</v>
       </c>
       <c r="K450">
-        <v>3.041971341412588</v>
+        <v>3.041971341412587</v>
       </c>
     </row>
     <row r="451" spans="1:11">
@@ -17332,10 +17332,10 @@
         <v>46181.3690625</v>
       </c>
       <c r="J473">
-        <v>1.842809472020499</v>
+        <v>1.8428094720205</v>
       </c>
       <c r="K473">
-        <v>1.842809472020499</v>
+        <v>1.8428094720205</v>
       </c>
     </row>
     <row r="474" spans="1:11">
@@ -18592,10 +18592,10 @@
         <v>46182.60833333333</v>
       </c>
       <c r="J509">
-        <v>2.502953491729752</v>
+        <v>2.502953491729751</v>
       </c>
       <c r="K509">
-        <v>2.502953491729752</v>
+        <v>2.502953491729751</v>
       </c>
     </row>
     <row r="510" spans="1:11">
@@ -19362,10 +19362,10 @@
         <v>46183.154375</v>
       </c>
       <c r="J531">
-        <v>2.645265851074053</v>
+        <v>2.645265851074052</v>
       </c>
       <c r="K531">
-        <v>2.645265851074053</v>
+        <v>2.645265851074052</v>
       </c>
     </row>
     <row r="532" spans="1:11">
@@ -19712,10 +19712,10 @@
         <v>46186.45532407407</v>
       </c>
       <c r="J541">
-        <v>1.551775839628436</v>
+        <v>1.551775839628435</v>
       </c>
       <c r="K541">
-        <v>1.551775839628436</v>
+        <v>1.551775839628435</v>
       </c>
     </row>
     <row r="542" spans="1:11">
@@ -20832,10 +20832,10 @@
         <v>46180.01618055555</v>
       </c>
       <c r="J573">
-        <v>1.614664383024041</v>
+        <v>1.61466438302404</v>
       </c>
       <c r="K573">
-        <v>1.614664383024041</v>
+        <v>1.61466438302404</v>
       </c>
     </row>
     <row r="574" spans="1:11">
@@ -21392,10 +21392,10 @@
         <v>46184.93923611111</v>
       </c>
       <c r="J589">
-        <v>4.690250207612562</v>
+        <v>4.690250207612561</v>
       </c>
       <c r="K589">
-        <v>4.690250207612562</v>
+        <v>4.690250207612561</v>
       </c>
     </row>
     <row r="590" spans="1:11">
@@ -21427,10 +21427,10 @@
         <v>46214.6469212963</v>
       </c>
       <c r="J590">
-        <v>4.481333785255095</v>
+        <v>4.481333785255094</v>
       </c>
       <c r="K590">
-        <v>4.481333785255095</v>
+        <v>4.481333785255094</v>
       </c>
     </row>
     <row r="591" spans="1:11">
@@ -21532,10 +21532,10 @@
         <v>46214.6469212963</v>
       </c>
       <c r="J593">
-        <v>4.481333785255095</v>
+        <v>4.481333785255094</v>
       </c>
       <c r="K593">
-        <v>4.481333785255095</v>
+        <v>4.481333785255094</v>
       </c>
     </row>
     <row r="594" spans="1:11">
@@ -21672,10 +21672,10 @@
         <v>46181.84710648148</v>
       </c>
       <c r="J597">
-        <v>4.999309442133119</v>
+        <v>4.99930944213312</v>
       </c>
       <c r="K597">
-        <v>4.999309442133119</v>
+        <v>4.99930944213312</v>
       </c>
     </row>
     <row r="598" spans="1:11">
@@ -21812,10 +21812,10 @@
         <v>46214.6469212963</v>
       </c>
       <c r="J601">
-        <v>6.264830902260329</v>
+        <v>6.26483090226033</v>
       </c>
       <c r="K601">
-        <v>6.264830902260329</v>
+        <v>6.26483090226033</v>
       </c>
     </row>
     <row r="602" spans="1:11">

</xml_diff>

<commit_message>
v3.2: feat - AOI_TT
</commit_message>
<xml_diff>
--- a/resources/M626/spc_cpk_detail.xlsx
+++ b/resources/M626/spc_cpk_detail.xlsx
@@ -775,10 +775,10 @@
         <v>46230.72840277778</v>
       </c>
       <c r="J2">
-        <v>1.783316479126941</v>
+        <v>1.783316479126942</v>
       </c>
       <c r="K2">
-        <v>1.783316479126941</v>
+        <v>1.783316479126942</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1090,10 +1090,10 @@
         <v>46238.89697916667</v>
       </c>
       <c r="J11">
-        <v>1.142303932752752</v>
+        <v>1.142303932752751</v>
       </c>
       <c r="K11">
-        <v>1.142303932752752</v>
+        <v>1.142303932752751</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1195,10 +1195,10 @@
         <v>46238.89697916667</v>
       </c>
       <c r="J14">
-        <v>1.142303932752752</v>
+        <v>1.142303932752751</v>
       </c>
       <c r="K14">
-        <v>1.142303932752752</v>
+        <v>1.142303932752751</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1300,10 +1300,10 @@
         <v>46238.89697916667</v>
       </c>
       <c r="J17">
-        <v>1.142303932752752</v>
+        <v>1.142303932752751</v>
       </c>
       <c r="K17">
-        <v>1.142303932752752</v>
+        <v>1.142303932752751</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -1650,10 +1650,10 @@
         <v>46239.94694444445</v>
       </c>
       <c r="J27">
-        <v>2.567108211495931</v>
+        <v>2.567108211495932</v>
       </c>
       <c r="K27">
-        <v>2.567108211495931</v>
+        <v>2.567108211495932</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2070,10 +2070,10 @@
         <v>46230.99207175926</v>
       </c>
       <c r="J39">
-        <v>2.066936758739829</v>
+        <v>2.066936758739828</v>
       </c>
       <c r="K39">
-        <v>2.066936758739829</v>
+        <v>2.066936758739828</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2595,10 +2595,10 @@
         <v>46240.07295138889</v>
       </c>
       <c r="J54">
-        <v>1.788942081069504</v>
+        <v>1.788942081069503</v>
       </c>
       <c r="K54">
-        <v>1.788942081069504</v>
+        <v>1.788942081069503</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -2665,10 +2665,10 @@
         <v>46240.07295138889</v>
       </c>
       <c r="J56">
-        <v>1.788942081069504</v>
+        <v>1.788942081069503</v>
       </c>
       <c r="K56">
-        <v>1.788942081069504</v>
+        <v>1.788942081069503</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -2735,10 +2735,10 @@
         <v>46240.07295138889</v>
       </c>
       <c r="J58">
-        <v>1.788942081069504</v>
+        <v>1.788942081069503</v>
       </c>
       <c r="K58">
-        <v>1.788942081069504</v>
+        <v>1.788942081069503</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -2980,10 +2980,10 @@
         <v>46240.72226851852</v>
       </c>
       <c r="J65">
-        <v>2.891429183460564</v>
+        <v>2.891429183460563</v>
       </c>
       <c r="K65">
-        <v>2.891429183460564</v>
+        <v>2.891429183460563</v>
       </c>
     </row>
     <row r="66" spans="1:11">
@@ -3505,10 +3505,10 @@
         <v>46233.92318287037</v>
       </c>
       <c r="J80">
-        <v>1.213053007796703</v>
+        <v>1.299305092733524</v>
       </c>
       <c r="K80">
-        <v>1.213053007796703</v>
+        <v>1.299305092733524</v>
       </c>
     </row>
     <row r="81" spans="1:11">
@@ -3540,10 +3540,10 @@
         <v>46241.44989583334</v>
       </c>
       <c r="J81">
-        <v>1.332850779869144</v>
+        <v>1.433809347294185</v>
       </c>
       <c r="K81">
-        <v>1.332850779869144</v>
+        <v>1.433809347294185</v>
       </c>
     </row>
     <row r="82" spans="1:11">
@@ -3575,10 +3575,10 @@
         <v>46233.92318287037</v>
       </c>
       <c r="J82">
-        <v>1.213053007796703</v>
+        <v>1.299305092733524</v>
       </c>
       <c r="K82">
-        <v>1.213053007796703</v>
+        <v>1.299305092733524</v>
       </c>
     </row>
     <row r="83" spans="1:11">
@@ -3610,10 +3610,10 @@
         <v>46241.44989583334</v>
       </c>
       <c r="J83">
-        <v>1.332850779869144</v>
+        <v>1.433809347294185</v>
       </c>
       <c r="K83">
-        <v>1.332850779869144</v>
+        <v>1.433809347294185</v>
       </c>
     </row>
     <row r="84" spans="1:11">
@@ -3645,10 +3645,10 @@
         <v>46233.92318287037</v>
       </c>
       <c r="J84">
-        <v>1.213053007796703</v>
+        <v>1.299305092733524</v>
       </c>
       <c r="K84">
-        <v>1.213053007796703</v>
+        <v>1.299305092733524</v>
       </c>
     </row>
     <row r="85" spans="1:11">
@@ -3680,10 +3680,10 @@
         <v>46241.44989583334</v>
       </c>
       <c r="J85">
-        <v>1.332850779869144</v>
+        <v>1.433809347294185</v>
       </c>
       <c r="K85">
-        <v>1.332850779869144</v>
+        <v>1.433809347294185</v>
       </c>
     </row>
     <row r="86" spans="1:11">
@@ -4205,10 +4205,10 @@
         <v>46238.68879629629</v>
       </c>
       <c r="J100">
-        <v>2.905559116600224</v>
+        <v>2.905559116600223</v>
       </c>
       <c r="K100">
-        <v>2.905559116600224</v>
+        <v>2.905559116600223</v>
       </c>
     </row>
     <row r="101" spans="1:11">
@@ -4345,10 +4345,10 @@
         <v>46238.74305555555</v>
       </c>
       <c r="J104">
-        <v>2.853604283911436</v>
+        <v>2.853604283911435</v>
       </c>
       <c r="K104">
-        <v>2.853604283911436</v>
+        <v>2.853604283911435</v>
       </c>
     </row>
     <row r="105" spans="1:11">
@@ -4555,10 +4555,10 @@
         <v>46242.52304398148</v>
       </c>
       <c r="J110">
-        <v>1.275138537961697</v>
+        <v>1.451262023593705</v>
       </c>
       <c r="K110">
-        <v>1.275138537961697</v>
+        <v>1.451262023593705</v>
       </c>
     </row>
     <row r="111" spans="1:11">
@@ -4590,10 +4590,10 @@
         <v>46242.52304398148</v>
       </c>
       <c r="J111">
-        <v>1.275138537961697</v>
+        <v>1.451262023593705</v>
       </c>
       <c r="K111">
-        <v>1.275138537961697</v>
+        <v>1.451262023593705</v>
       </c>
     </row>
     <row r="112" spans="1:11">
@@ -4625,10 +4625,10 @@
         <v>46238.74305555555</v>
       </c>
       <c r="J112">
-        <v>1.199874216297309</v>
+        <v>1.358568807624723</v>
       </c>
       <c r="K112">
-        <v>1.199874216297309</v>
+        <v>1.358568807624723</v>
       </c>
     </row>
     <row r="113" spans="1:11">
@@ -4660,10 +4660,10 @@
         <v>46242.52304398148</v>
       </c>
       <c r="J113">
-        <v>1.337787016703079</v>
+        <v>1.490845501850582</v>
       </c>
       <c r="K113">
-        <v>1.337787016703079</v>
+        <v>1.490845501850582</v>
       </c>
     </row>
     <row r="114" spans="1:11">
@@ -4905,10 +4905,10 @@
         <v>46237.2683912037</v>
       </c>
       <c r="J120">
-        <v>1.683802188892684</v>
+        <v>1.683802188892685</v>
       </c>
       <c r="K120">
-        <v>1.683802188892684</v>
+        <v>1.683802188892685</v>
       </c>
     </row>
     <row r="121" spans="1:11">
@@ -4940,10 +4940,10 @@
         <v>46240.58334490741</v>
       </c>
       <c r="J121">
-        <v>1.476682718879129</v>
+        <v>1.476682718879128</v>
       </c>
       <c r="K121">
-        <v>1.476682718879129</v>
+        <v>1.476682718879128</v>
       </c>
     </row>
     <row r="122" spans="1:11">
@@ -5360,10 +5360,10 @@
         <v>46240.66833333333</v>
       </c>
       <c r="J133">
-        <v>1.895099538835158</v>
+        <v>1.895099538835159</v>
       </c>
       <c r="K133">
-        <v>1.895099538835158</v>
+        <v>1.895099538835159</v>
       </c>
     </row>
     <row r="134" spans="1:11">
@@ -5395,10 +5395,10 @@
         <v>46242.51028935185</v>
       </c>
       <c r="J134">
-        <v>1.232890123162044</v>
+        <v>1.232890123162045</v>
       </c>
       <c r="K134">
-        <v>1.232890123162044</v>
+        <v>1.232890123162045</v>
       </c>
     </row>
     <row r="135" spans="1:11">
@@ -5885,10 +5885,10 @@
         <v>46243.8480787037</v>
       </c>
       <c r="J148">
-        <v>1.250385759207341</v>
+        <v>1.362323444544703</v>
       </c>
       <c r="K148">
-        <v>1.250385759207341</v>
+        <v>1.362323444544703</v>
       </c>
     </row>
     <row r="149" spans="1:11">
@@ -5920,10 +5920,10 @@
         <v>46243.8480787037</v>
       </c>
       <c r="J149">
-        <v>1.250385759207341</v>
+        <v>1.362323444544703</v>
       </c>
       <c r="K149">
-        <v>1.250385759207341</v>
+        <v>1.362323444544703</v>
       </c>
     </row>
     <row r="150" spans="1:11">
@@ -5955,10 +5955,10 @@
         <v>46243.8480787037</v>
       </c>
       <c r="J150">
-        <v>1.250385759207341</v>
+        <v>1.362323444544703</v>
       </c>
       <c r="K150">
-        <v>1.250385759207341</v>
+        <v>1.362323444544703</v>
       </c>
     </row>
     <row r="151" spans="1:11">
@@ -7530,10 +7530,10 @@
         <v>46237.40302083334</v>
       </c>
       <c r="J195">
-        <v>1.699841446416683</v>
+        <v>1.699841446416682</v>
       </c>
       <c r="K195">
-        <v>1.699841446416683</v>
+        <v>1.699841446416682</v>
       </c>
     </row>
     <row r="196" spans="1:11">
@@ -8195,10 +8195,10 @@
         <v>46207.44892361111</v>
       </c>
       <c r="J214">
-        <v>1.978853450574099</v>
+        <v>1.978853450574098</v>
       </c>
       <c r="K214">
-        <v>1.978853450574099</v>
+        <v>1.978853450574098</v>
       </c>
     </row>
     <row r="215" spans="1:11">
@@ -8230,10 +8230,10 @@
         <v>46207.44892361111</v>
       </c>
       <c r="J215">
-        <v>1.978853450574099</v>
+        <v>1.978853450574098</v>
       </c>
       <c r="K215">
-        <v>1.978853450574099</v>
+        <v>1.978853450574098</v>
       </c>
     </row>
     <row r="216" spans="1:11">
@@ -8720,10 +8720,10 @@
         <v>46205.77965277778</v>
       </c>
       <c r="J229">
-        <v>2.013994314162455</v>
+        <v>2.013994314162456</v>
       </c>
       <c r="K229">
-        <v>2.013994314162455</v>
+        <v>2.013994314162456</v>
       </c>
     </row>
     <row r="230" spans="1:11">
@@ -8895,10 +8895,10 @@
         <v>46204.48143518518</v>
       </c>
       <c r="J234">
-        <v>5.266814649998149</v>
+        <v>5.26681464999815</v>
       </c>
       <c r="K234">
-        <v>5.266814649998149</v>
+        <v>5.26681464999815</v>
       </c>
     </row>
     <row r="235" spans="1:11">
@@ -9560,10 +9560,10 @@
         <v>46205.74839120371</v>
       </c>
       <c r="J253">
-        <v>5.850465480446285</v>
+        <v>5.850465480446287</v>
       </c>
       <c r="K253">
-        <v>5.850465480446285</v>
+        <v>5.850465480446287</v>
       </c>
     </row>
     <row r="254" spans="1:11">
@@ -9805,10 +9805,10 @@
         <v>46206.66802083333</v>
       </c>
       <c r="J260">
-        <v>3.078750218465228</v>
+        <v>3.078750218465227</v>
       </c>
       <c r="K260">
-        <v>3.078750218465228</v>
+        <v>3.078750218465227</v>
       </c>
     </row>
     <row r="261" spans="1:11">
@@ -10505,10 +10505,10 @@
         <v>46207.23274305555</v>
       </c>
       <c r="J280">
-        <v>1.990153757485192</v>
+        <v>1.990153757485191</v>
       </c>
       <c r="K280">
-        <v>1.990153757485192</v>
+        <v>1.990153757485191</v>
       </c>
     </row>
     <row r="281" spans="1:11">
@@ -10540,10 +10540,10 @@
         <v>46207.23274305555</v>
       </c>
       <c r="J281">
-        <v>1.990153757485192</v>
+        <v>1.990153757485191</v>
       </c>
       <c r="K281">
-        <v>1.990153757485192</v>
+        <v>1.990153757485191</v>
       </c>
     </row>
     <row r="282" spans="1:11">
@@ -10575,10 +10575,10 @@
         <v>46207.23274305555</v>
       </c>
       <c r="J282">
-        <v>1.990153757485192</v>
+        <v>1.990153757485191</v>
       </c>
       <c r="K282">
-        <v>1.990153757485192</v>
+        <v>1.990153757485191</v>
       </c>
     </row>
     <row r="283" spans="1:11">
@@ -11695,10 +11695,10 @@
         <v>46209.56375</v>
       </c>
       <c r="J314">
-        <v>4.852419037731009</v>
+        <v>4.85241903773101</v>
       </c>
       <c r="K314">
-        <v>4.852419037731009</v>
+        <v>4.85241903773101</v>
       </c>
     </row>
     <row r="315" spans="1:11">
@@ -11870,10 +11870,10 @@
         <v>46209.95513888889</v>
       </c>
       <c r="J319">
-        <v>1.886380431790312</v>
+        <v>1.886380431790313</v>
       </c>
       <c r="K319">
-        <v>1.886380431790312</v>
+        <v>1.886380431790313</v>
       </c>
     </row>
     <row r="320" spans="1:11">

</xml_diff>